<commit_message>
fix(wifi_llapi): 修正 Summary 待確認統計與通過率
- 將 Summary 顯示 bucket 從 To be tested 改為 To be confirmed
- 將 Summary Pass Rate 公式改為只計算 Pass / (Pass + Fail)
- 強化 template validation 拒絕舊 bucket 文字與 E:G 通過率公式
- 更新 template 說明文字、報表輸出標籤與回歸測試

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/plugins/wifi_llapi/reports/templates/wifi_llapi_template.xlsx
+++ b/plugins/wifi_llapi/reports/templates/wifi_llapi_template.xlsx
@@ -1777,7 +1777,7 @@
       </c>
       <c r="G2" s="171" t="inlineStr">
         <is>
-          <t>To be tested</t>
+          <t>To be confirmed</t>
         </is>
       </c>
       <c r="H2" s="171" t="inlineStr">
@@ -1846,7 +1846,7 @@
         <v/>
       </c>
       <c r="J3" s="155">
-        <f>IFERROR(E3/SUM(E3:G3),0)</f>
+        <f>IFERROR(E3/SUM(E3:F3),0)</f>
         <v/>
       </c>
       <c r="K3" s="140">
@@ -1909,7 +1909,7 @@
         <v/>
       </c>
       <c r="J4" s="150">
-        <f>IFERROR(E4/SUM(E4:G4),0)</f>
+        <f>IFERROR(E4/SUM(E4:F4),0)</f>
         <v/>
       </c>
       <c r="K4" s="140">
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="J5" s="150">
-        <f>IFERROR(E5/SUM(E5:G5),0)</f>
+        <f>IFERROR(E5/SUM(E5:F5),0)</f>
         <v/>
       </c>
       <c r="K5" s="140">
@@ -2029,7 +2029,7 @@
         <v/>
       </c>
       <c r="J6" s="150">
-        <f>IFERROR(E6/SUM(E6:G6),0)</f>
+        <f>IFERROR(E6/SUM(E6:F6),0)</f>
         <v/>
       </c>
       <c r="K6" s="140">
@@ -2089,7 +2089,7 @@
         <v/>
       </c>
       <c r="J7" s="150">
-        <f>IFERROR(E7/SUM(E7:G7),0)</f>
+        <f>IFERROR(E7/SUM(E7:F7),0)</f>
         <v/>
       </c>
       <c r="K7" s="140">
@@ -2137,7 +2137,7 @@
         <v/>
       </c>
       <c r="J8" s="146">
-        <f>IFERROR(E8/SUM(E8:G8),0)</f>
+        <f>IFERROR(E8/SUM(E8:F8),0)</f>
         <v/>
       </c>
       <c r="K8" s="145">
@@ -2189,7 +2189,7 @@
         <v/>
       </c>
       <c r="J9" s="155">
-        <f>IFERROR(E9/SUM(E9:G9),0)</f>
+        <f>IFERROR(E9/SUM(E9:F9),0)</f>
         <v/>
       </c>
       <c r="K9" s="140">
@@ -2237,7 +2237,7 @@
         <v/>
       </c>
       <c r="J10" s="150">
-        <f>IFERROR(E10/SUM(E10:G10),0)</f>
+        <f>IFERROR(E10/SUM(E10:F10),0)</f>
         <v/>
       </c>
       <c r="K10" s="140">
@@ -2285,7 +2285,7 @@
         <v/>
       </c>
       <c r="J11" s="150">
-        <f>IFERROR(E11/SUM(E11:G11),0)</f>
+        <f>IFERROR(E11/SUM(E11:F11),0)</f>
         <v/>
       </c>
       <c r="K11" s="140">
@@ -2333,7 +2333,7 @@
         <v/>
       </c>
       <c r="J12" s="150">
-        <f>IFERROR(E12/SUM(E12:G12),0)</f>
+        <f>IFERROR(E12/SUM(E12:F12),0)</f>
         <v/>
       </c>
       <c r="K12" s="140">
@@ -2381,7 +2381,7 @@
         <v/>
       </c>
       <c r="J13" s="150">
-        <f>IFERROR(E13/SUM(E13:G13),0)</f>
+        <f>IFERROR(E13/SUM(E13:F13),0)</f>
         <v/>
       </c>
       <c r="K13" s="140">
@@ -2429,7 +2429,7 @@
         <v/>
       </c>
       <c r="J14" s="146">
-        <f>IFERROR(E14/SUM(E14:G14),0)</f>
+        <f>IFERROR(E14/SUM(E14:F14),0)</f>
         <v/>
       </c>
       <c r="K14" s="145">
@@ -2481,7 +2481,7 @@
         <v/>
       </c>
       <c r="J15" s="155">
-        <f>IFERROR(E15/SUM(E15:G15),0)</f>
+        <f>IFERROR(E15/SUM(E15:F15),0)</f>
         <v/>
       </c>
       <c r="K15" s="140">
@@ -2529,7 +2529,7 @@
         <v/>
       </c>
       <c r="J16" s="150">
-        <f>IFERROR(E16/SUM(E16:G16),0)</f>
+        <f>IFERROR(E16/SUM(E16:F16),0)</f>
         <v/>
       </c>
       <c r="K16" s="140">
@@ -2577,7 +2577,7 @@
         <v/>
       </c>
       <c r="J17" s="150">
-        <f>IFERROR(E17/SUM(E17:G17),0)</f>
+        <f>IFERROR(E17/SUM(E17:F17),0)</f>
         <v/>
       </c>
       <c r="K17" s="140">
@@ -2625,7 +2625,7 @@
         <v/>
       </c>
       <c r="J18" s="150">
-        <f>IFERROR(E18/SUM(E18:G18),0)</f>
+        <f>IFERROR(E18/SUM(E18:F18),0)</f>
         <v/>
       </c>
       <c r="K18" s="140">
@@ -2673,7 +2673,7 @@
         <v/>
       </c>
       <c r="J19" s="150">
-        <f>IFERROR(E19/SUM(E19:G19),0)</f>
+        <f>IFERROR(E19/SUM(E19:F19),0)</f>
         <v/>
       </c>
       <c r="K19" s="140">
@@ -2721,7 +2721,7 @@
         <v/>
       </c>
       <c r="J20" s="146">
-        <f>IFERROR(E20/SUM(E20:G20),0)</f>
+        <f>IFERROR(E20/SUM(E20:F20),0)</f>
         <v/>
       </c>
       <c r="K20" s="145">
@@ -2739,12 +2739,12 @@
         <is>
           <t>Total Items : 
 The total number of test items defined for the object category. The total value include. 
-The value of Total Items is the sum of Pass, Fail, To be tested, Not Supported, and Skip items.
+The value of Total Items is the sum of Pass, Fail, To be confirmed, Not Supported, and Skip items.
 Pass : 
 Tested and passed
 Fail : 
 Tested and failed
-To be tested:
+To be confirmed:
 1. In the current test environment, no Wi-Fi station is capable of generating intentionally malformed or manipulated IEEE 802.11e error frames. Additionally, Scapy cannot be used for this purpose due to Wi-Fi station and driver limitations.
 Testing will be revisited once appropriate Wi-Fi protocol test equipment or interference generation capability becomes available.
 2. No ethernet RMON test environment
@@ -2754,7 +2754,7 @@
 Skip : 
 This project is a gateway (GW) and does not support WiFi Station Mode.
 Pass Rate : 
-The percentage of passed test items, calculated as Pass / (Pass + Fail + To be tested).</t>
+The percentage of passed test items, calculated as Pass / (Pass + Fail).</t>
         </is>
       </c>
     </row>
@@ -2968,17 +2968,17 @@
           <t>Comment</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="0" t="inlineStr">
         <is>
           <t>Summary Bucket WiFi 5G</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="0" t="inlineStr">
         <is>
           <t>Summary Bucket WiFi 6G</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" s="0" t="inlineStr">
         <is>
           <t>Summary Bucket WiFi 2.4G</t>
         </is>

</xml_diff>